<commit_message>
data: cierre dia 2026-10-01_1749 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/OBJSELLOUT.xlsx
+++ b/01_INPUTS/OBJSELLOUT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Orbit\MATINAL_PENAFLOR\01_INPUTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B72A0308-DBA3-46B6-8EA6-004008EC1AAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1DAE6F7-AD2C-4B0C-A787-F6044697F9D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -263,32 +263,32 @@
     <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="1" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -612,11 +612,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="14"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="21"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -637,7 +637,7 @@
         <v>5</v>
       </c>
       <c r="C3" s="11">
-        <v>13217.150326380846</v>
+        <v>12338.254394006195</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -647,8 +647,8 @@
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="18">
-        <v>365.15940424038524</v>
+      <c r="C4" s="15">
+        <v>364.57265456228157</v>
       </c>
       <c r="D4" s="1"/>
     </row>
@@ -659,8 +659,8 @@
       <c r="B5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="18">
-        <v>4462.8536073903924</v>
+      <c r="C5" s="15">
+        <v>4423.6250176998237</v>
       </c>
       <c r="D5" s="1"/>
     </row>
@@ -671,8 +671,8 @@
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="18">
-        <v>2466.3693174301065</v>
+      <c r="C6" s="15">
+        <v>2200.3180020012956</v>
       </c>
       <c r="D6" s="1"/>
     </row>
@@ -685,7 +685,7 @@
       </c>
       <c r="C7" s="11">
         <f>SUM(C3:C6)</f>
-        <v>20511.532655441733</v>
+        <v>19326.770068269594</v>
       </c>
       <c r="D7" s="1"/>
     </row>
@@ -696,8 +696,8 @@
       <c r="B8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="20">
-        <v>1372.2704956991149</v>
+      <c r="C8" s="17">
+        <v>692.35942389825175</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -707,8 +707,8 @@
       <c r="B9" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="17">
-        <v>489.01923646361087</v>
+      <c r="C9" s="14">
+        <v>399.07461890724556</v>
       </c>
       <c r="D9" s="1"/>
     </row>
@@ -719,8 +719,8 @@
       <c r="B10" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="17">
-        <v>26540.575745363996</v>
+      <c r="C10" s="14">
+        <v>24924.760539399191</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -730,9 +730,9 @@
       <c r="B11" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="17">
+      <c r="C11" s="14">
         <f>SUM(C9:C10)</f>
-        <v>27029.594981827606</v>
+        <v>25323.835158306436</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -742,7 +742,7 @@
       <c r="B12" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="19"/>
+      <c r="C12" s="16"/>
       <c r="D12" s="10"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -762,8 +762,8 @@
       <c r="B14" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="19">
-        <v>14543.321694671846</v>
+      <c r="C14" s="16">
+        <v>16418.049284201865</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -773,8 +773,8 @@
       <c r="B15" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="16">
-        <v>1478.3740365045551</v>
+      <c r="C15" s="13">
+        <v>4754.2063211815557</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -784,8 +784,8 @@
       <c r="B16" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="15">
-        <v>656.55243169487835</v>
+      <c r="C16" s="12">
+        <v>699.1806169495668</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -795,8 +795,8 @@
       <c r="B17" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="20">
-        <v>6346.5261243215537</v>
+      <c r="C17" s="17">
+        <v>6970.3517832180578</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -804,8 +804,9 @@
         <v>21</v>
       </c>
       <c r="B18" s="9"/>
-      <c r="C18" s="21">
-        <v>71938.172420161281</v>
+      <c r="C18" s="18">
+        <f>SUM(C7,C8,C11,C14,C15,C16,C17)</f>
+        <v>74184.752656025332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>